<commit_message>
update and first results
</commit_message>
<xml_diff>
--- a/latex/tabs/algorithm_comparison.xlsx
+++ b/latex/tabs/algorithm_comparison.xlsx
@@ -458,20 +458,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BaselineOnly</t>
+          <t>SVD</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7492012818406858</v>
+        <v>0.6571</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6036991240262529</v>
+        <v>0.5286999999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>0.5614235123496866</v>
+        <v>0.4319</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5101231898504396</v>
+        <v>0.5436</v>
       </c>
     </row>
     <row r="3">
@@ -481,54 +481,54 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9288444549060079</v>
+        <v>1.181</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8103420761955668</v>
+        <v>0.9747</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8627530273104528</v>
+        <v>1.3948</v>
       </c>
       <c r="E3" t="n">
-        <v>0.437115674340361</v>
+        <v>0.5568</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NMF</t>
+          <t>BaselineOnly</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7785668259574151</v>
+        <v>0.6552</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6284678283403711</v>
+        <v>0.538</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6061720817216799</v>
+        <v>0.4293</v>
       </c>
       <c r="E4" t="n">
-        <v>0.506355236236821</v>
+        <v>0.5686</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SVD</t>
+          <t>NMF</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.7513082874111404</v>
+        <v>0.8391999999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>0.5992514557717208</v>
+        <v>0.6342</v>
       </c>
       <c r="D5" t="n">
-        <v>0.56470932030174</v>
+        <v>0.7043</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5160281241267252</v>
+        <v>0.4964</v>
       </c>
     </row>
   </sheetData>

</xml_diff>